<commit_message>
change for 5 lecture
</commit_message>
<xml_diff>
--- a/Lecture5.Agents/data/evaluation_dataset.xlsx
+++ b/Lecture5.Agents/data/evaluation_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleksandrmeskov/Desktop/AI evaluation/AI_practice/Lecture6/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aleksandrmeskov/Projects/Evaluation_AI_course_eng/Lecture5.Agents/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A690CE47-35CF-D14E-8739-D536FBD9972D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99683B8B-E5E8-DE48-B891-32E9D85FB10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10360" yWindow="1720" windowWidth="28040" windowHeight="17440" xr2:uid="{BF369E15-F991-6B4A-BC00-4B14A4CF84E4}"/>
   </bookViews>
@@ -47,16 +47,16 @@
     <t>expected_tools</t>
   </si>
   <si>
-    <t>Найди квартиры дешевле 3000 долларов</t>
-  </si>
-  <si>
     <t>extract_offers, filter_offers</t>
   </si>
   <si>
-    <t>Найди квартиры дешевле 3000 долларов и конвертируй их в рубли</t>
-  </si>
-  <si>
     <t>extract_offers, normalize_offers_currency</t>
+  </si>
+  <si>
+    <t>Find apartments cheaper than 3000 dollars</t>
+  </si>
+  <si>
+    <t>Find apartments cheaper than 3000 dollars and convert prices to euros</t>
   </si>
 </sst>
 </file>
@@ -466,18 +466,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>